<commit_message>
decide on some data values
</commit_message>
<xml_diff>
--- a/0100_data_prep/extraction/LSFF_effect_sizes.xlsx
+++ b/0100_data_prep/extraction/LSFF_effect_sizes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30601"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid.sharepoint.com/sites/ihme_simulation_science_team/Shared Documents/Research/LSFF/Phase 3 (2026-2027)/Literature/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4BB281B6-C202-4DAC-B00B-ECC885F85582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D4AE21D5-5DA4-4C16-B664-951AE866AC97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" firstSheet="3" activeTab="3" xr2:uid="{E4FDD644-5F65-E746-9A1B-54C2B87A6AA0}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" firstSheet="3" activeTab="4" xr2:uid="{E4FDD644-5F65-E746-9A1B-54C2B87A6AA0}"/>
   </bookViews>
   <sheets>
     <sheet name="Fortification" sheetId="1" r:id="rId1"/>
@@ -11912,7 +11912,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="31.15">
+    <row r="5" spans="1:10" ht="30.75">
       <c r="A5" s="3" t="s">
         <v>336</v>
       </c>
@@ -11923,7 +11923,7 @@
         <v>298</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>121</v>
+        <v>332</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>337</v>
@@ -11944,7 +11944,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="31.15">
+    <row r="6" spans="1:10" ht="30.75">
       <c r="A6" s="3" t="s">
         <v>336</v>
       </c>
@@ -11955,7 +11955,7 @@
         <v>321</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>121</v>
+        <v>332</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>337</v>
@@ -11976,7 +11976,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" ht="15.75">
       <c r="A7" s="3" t="s">
         <v>336</v>
       </c>
@@ -11987,7 +11987,7 @@
         <v>321</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>121</v>
+        <v>332</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>337</v>

</xml_diff>